<commit_message>
Leva 1: núcleo de auditoria corrigido
Itens aplicados em Auditoria interna, Técnica de auditoria, Processo de
certificação e Não conformidade:
- T01, T02, T03, T04: um desvio com evidência objetiva já é não
  conformidade; a não conformidade pede ao menos uma fonte objetiva
  (fórmulas, rótulos e painel da planilha de Técnica, testes da planilha).
- T05: constatação 3 da auditoria 2026-03 passa a NC menor.
- T06: verificação por quem não executou as ações passa a "convém".
- I01 (Auditoria, exemplo 3), I03 (Certificação, I-3, figura e questionário).
- D08: frase padrão nos "Pontos de atenção" do módulo das normas.
- Decisões da ficha: P09, N02, N18, N20, N22.
- N23 (novo em DECISOES): propagação de T05 para a análise crítica (c4 e
  c6) e para Competências.
- Regras novas em PROIBIDO: T01, T02b, T03, T04, T05, T06, N02, N20, N22a,
  P09a.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Analise-Critica/Analise-Critica-modelo.xlsx
+++ b/Analise-Critica/Analise-Critica-modelo.xlsx
@@ -1156,7 +1156,7 @@
     <t xml:space="preserve">O sistema cobre bem o delivery, e pouco o restante da loja.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dois registros no ano, os dois da auditoria 2026-03. O RNC 2026-05 foi encerrado como eficaz. O segundo está em verificação.</t>
+    <t xml:space="preserve">Três registros abertos pela auditoria 2026-03. O RNC 2026-05 foi encerrado como eficaz. Os outros dois estão em verificação.</t>
   </si>
   <si>
     <t xml:space="preserve">O tratamento funciona. Manter.</t>
@@ -1171,7 +1171,7 @@
     <t xml:space="preserve">As medições são feitas e usadas. Manter.</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma auditoria no ano, no delivery: duas não conformidades menores e uma oportunidade de melhoria. O salão e as compras nunca foram auditados.</t>
+    <t xml:space="preserve">A auditoria 2026-03, no delivery: três não conformidades menores. O salão e as compras nunca foram auditados.</t>
   </si>
   <si>
     <t xml:space="preserve">O programa de auditoria precisa cobrir os outros processos.</t>
@@ -2194,11 +2194,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="66066051"/>
-        <c:axId val="34742486"/>
+        <c:axId val="96490303"/>
+        <c:axId val="35167514"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="66066051"/>
+        <c:axId val="96490303"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2230,7 +2230,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34742486"/>
+        <c:crossAx val="35167514"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2238,7 +2238,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34742486"/>
+        <c:axId val="35167514"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2278,7 +2278,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66066051"/>
+        <c:crossAx val="96490303"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -2420,11 +2420,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="33181274"/>
-        <c:axId val="96108305"/>
+        <c:axId val="50633389"/>
+        <c:axId val="46297849"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="33181274"/>
+        <c:axId val="50633389"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2456,7 +2456,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96108305"/>
+        <c:crossAx val="46297849"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2464,7 +2464,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="96108305"/>
+        <c:axId val="46297849"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2504,7 +2504,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33181274"/>
+        <c:crossAx val="50633389"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -5430,16 +5430,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H21" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Item da entrada: a, b, c1 a c7, d, e ou f" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7:C21" type="list">
       <formula1>"a,b,c1,c2,c3,c4,c5,c6,c7,d,e,f"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Melhoria, Mudança no sistema ou Recursos" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E7:E21" type="list">
       <formula1>"Melhoria,Mudança no sistema,Recursos"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H21" type="date">
+      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Digite apenas o número, sem texto nem unidade." errorStyle="stop" errorTitle="Valor inválido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J7:J21" type="decimal">

</xml_diff>